<commit_message>
Ajusta referências da planilha de conteúdo da Imersão DPM
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqFY5sbivnPXvpYHTJ29PX
</commit_message>
<xml_diff>
--- a/imersao-dpm/planilha/planejamento-conteudo-imersao-dpm.xlsx
+++ b/imersao-dpm/planilha/planejamento-conteudo-imersao-dpm.xlsx
@@ -526,7 +526,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Abertura · Material de Apoio p.6 · PDF Aula 01 p.2</t>
+          <t>Noite 1 · Abertura · Material de Apoio p.6 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -588,7 +588,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição I · Material de Apoio p.6 · PDF Aula 01 p.3</t>
+          <t>Noite 1 · Lição I · Material de Apoio p.6 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição II · Material de Apoio p.6-7 · PDF Aula 01 p.3</t>
+          <t>Noite 1 · Lição II · Material de Apoio p.6-7 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição III · Material de Apoio p.7 · PDF Aula 01 p.4</t>
+          <t>Noite 1 · Lição III · Material de Apoio p.7 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição IV · Material de Apoio p.7 · PDF Aula 01 p.4</t>
+          <t>Noite 1 · Lição IV · Material de Apoio p.7 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição IV · Material de Apoio p.7 · PDF Aula 01 p.4</t>
+          <t>Noite 1 · Lição IV · Material de Apoio p.7 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição V · Material de Apoio p.8 · PDF Aula 01 p.5</t>
+          <t>Noite 1 · Lição V · Material de Apoio p.8 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição VI · Material de Apoio p.8-9 · PDF Aula 01 p.6</t>
+          <t>Noite 1 · Lição VI · Material de Apoio p.8-9 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Abertura · Material de Apoio p.13 · PDF Aula 02 p.2</t>
+          <t>Noite 2 · Abertura · Material de Apoio p.13 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Lição I · Material de Apoio p.13 · PDF Aula 02 p.3</t>
+          <t>Noite 2 · Lição I · Material de Apoio p.13 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Lição II · Material de Apoio p.13-14 · PDF Aula 02 p.3</t>
+          <t>Noite 2 · Lição II · Material de Apoio p.13-14 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Lição V · Material de Apoio p.14-15 · PDF Aula 02 p.4</t>
+          <t>Noite 2 · Lição V · Material de Apoio p.14-15 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Prática · Material de Apoio p.16-17 · PDF Aula 02 p.5</t>
+          <t>Noite 2 · Prática · Material de Apoio p.16-17 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Não trave o processo · Material de Apoio p.17 · PDF Aula 02 p.6</t>
+          <t>Noite 2 · Não trave o processo · Material de Apoio p.17 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Noite 3 · Abertura · Material de Apoio p.20 · PDF Aula 03 p.2</t>
+          <t>Noite 3 · Abertura · Material de Apoio p.20 · PDF Aula 03</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Noite 3 · Eu do futuro · Material de Apoio p.22 · PDF Aula 03 p.4</t>
+          <t>Noite 3 · Eu do futuro · Material de Apoio p.22 · PDF Aula 03</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lições I a IV · Material de Apoio p.6-7 · PDF Aula 01 p.3-4</t>
+          <t>Noite 1 · Lições I a IV · Material de Apoio p.6-7 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição VI · Material de Apoio p.8-9 · PDF Aula 01 p.6</t>
+          <t>Noite 1 · Lição VI · Material de Apoio p.8-9 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Lição IV · Material de Apoio p.14 · PDF Aula 02 p.4</t>
+          <t>Noite 2 · Lição IV · Material de Apoio p.14 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Lições II e III · Material de Apoio p.13-14 · PDF Aula 02 p.3</t>
+          <t>Noite 2 · Lições II e III · Material de Apoio p.13-14 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Lição VI · Material de Apoio p.15 · PDF Aula 02 p.5</t>
+          <t>Noite 2 · Lição VI · Material de Apoio p.15 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Prática · Material de Apoio p.17 · PDF Aula 02 p.5</t>
+          <t>Noite 2 · Prática · Material de Apoio p.17 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Noite 3 · Exercícios 1 e 2 · Material de Apoio p.20-21 · PDF Aula 03 p.3-4</t>
+          <t>Noite 3 · Exercícios 1 e 2 · Material de Apoio p.20-21 · PDF Aula 03</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1952,7 +1952,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Rotina · Material de Apoio p.26 · PDF Aula 03 p.7</t>
+          <t>Rotina · Material de Apoio p.26 · PDF Aula 03</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Exercício · Material de Apoio p.9-10 · PDF Aula 01 p.7</t>
+          <t>Noite 1 · Exercício · Material de Apoio p.9-10 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Abertura · Material de Apoio p.6 · PDF Aula 01 p.2</t>
+          <t>Noite 1 · Abertura · Material de Apoio p.6 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição I · Material de Apoio p.6 · PDF Aula 01 p.3</t>
+          <t>Noite 1 · Lição I · Material de Apoio p.6 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição II · Material de Apoio p.6-7 · PDF Aula 01 p.3</t>
+          <t>Noite 1 · Lição II · Material de Apoio p.6-7 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -3282,7 +3282,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição III · Material de Apoio p.7 · PDF Aula 01 p.4</t>
+          <t>Noite 1 · Lição III · Material de Apoio p.7 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição IV · Material de Apoio p.7 · PDF Aula 01 p.4</t>
+          <t>Noite 1 · Lição IV · Material de Apoio p.7 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição IV · Material de Apoio p.7 · PDF Aula 01 p.4</t>
+          <t>Noite 1 · Lição IV · Material de Apoio p.7 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição V · Material de Apoio p.8 · PDF Aula 01 p.5</t>
+          <t>Noite 1 · Lição V · Material de Apoio p.8 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -3530,7 +3530,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição VI · Material de Apoio p.8-9 · PDF Aula 01 p.6</t>
+          <t>Noite 1 · Lição VI · Material de Apoio p.8-9 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -3592,7 +3592,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Abertura · Material de Apoio p.13 · PDF Aula 02 p.2</t>
+          <t>Noite 2 · Abertura · Material de Apoio p.13 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Lição I · Material de Apoio p.13 · PDF Aula 02 p.3</t>
+          <t>Noite 2 · Lição I · Material de Apoio p.13 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -3716,7 +3716,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Lição II · Material de Apoio p.13-14 · PDF Aula 02 p.3</t>
+          <t>Noite 2 · Lição II · Material de Apoio p.13-14 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -3778,7 +3778,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Lição V · Material de Apoio p.14-15 · PDF Aula 02 p.4</t>
+          <t>Noite 2 · Lição V · Material de Apoio p.14-15 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Prática · Material de Apoio p.16-17 · PDF Aula 02 p.5</t>
+          <t>Noite 2 · Prática · Material de Apoio p.16-17 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -3902,7 +3902,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Não trave o processo · Material de Apoio p.17 · PDF Aula 02 p.6</t>
+          <t>Noite 2 · Não trave o processo · Material de Apoio p.17 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Noite 3 · Abertura · Material de Apoio p.20 · PDF Aula 03 p.2</t>
+          <t>Noite 3 · Abertura · Material de Apoio p.20 · PDF Aula 03</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Noite 3 · Eu do futuro · Material de Apoio p.22 · PDF Aula 03 p.4</t>
+          <t>Noite 3 · Eu do futuro · Material de Apoio p.22 · PDF Aula 03</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lições I a IV · Material de Apoio p.6-7 · PDF Aula 01 p.3-4</t>
+          <t>Noite 1 · Lições I a IV · Material de Apoio p.6-7 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Lição VI · Material de Apoio p.8-9 · PDF Aula 01 p.6</t>
+          <t>Noite 1 · Lição VI · Material de Apoio p.8-9 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -4302,7 +4302,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Lição IV · Material de Apoio p.14 · PDF Aula 02 p.4</t>
+          <t>Noite 2 · Lição IV · Material de Apoio p.14 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Lições II e III · Material de Apoio p.13-14 · PDF Aula 02 p.3</t>
+          <t>Noite 2 · Lições II e III · Material de Apoio p.13-14 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Lição VI · Material de Apoio p.15 · PDF Aula 02 p.5</t>
+          <t>Noite 2 · Lição VI · Material de Apoio p.15 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -4488,7 +4488,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Noite 2 · Prática · Material de Apoio p.17 · PDF Aula 02 p.5</t>
+          <t>Noite 2 · Prática · Material de Apoio p.17 · PDF Aula 02</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Noite 3 · Exercícios 1 e 2 · Material de Apoio p.20-21 · PDF Aula 03 p.3-4</t>
+          <t>Noite 3 · Exercícios 1 e 2 · Material de Apoio p.20-21 · PDF Aula 03</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -4612,7 +4612,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Rotina · Material de Apoio p.26 · PDF Aula 03 p.7</t>
+          <t>Rotina · Material de Apoio p.26 · PDF Aula 03</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -4950,7 +4950,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Noite 1 · Exercício · Material de Apoio p.9-10 · PDF Aula 01 p.7</t>
+          <t>Noite 1 · Exercício · Material de Apoio p.9-10 · PDF Aula 01</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">

</xml_diff>